<commit_message>
feat: restaurar articulo PP19568-02 al catalogo maestro (eliminado por error en actualizacion masiva)
</commit_message>
<xml_diff>
--- a/BD_Articulos.xlsx
+++ b/BD_Articulos.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Datos_Sistema" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Datos_Sistema" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E124"/>
+  <dimension ref="A1:E125"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3764,6 +3764,33 @@
         </is>
       </c>
     </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>PP19568-02</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>PP19568-02-(16gacr ANSI-61) - K48 - V1-R0</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>16GACR</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>Length: 16.22 * Width: 36.09</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>Ansi 61</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: actualizar catalogo BD_Articulos con 126 SKUs cliente reales y eliminar prefijo provisional CLI-
</commit_message>
<xml_diff>
--- a/BD_Articulos.xlsx
+++ b/BD_Articulos.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1065" uniqueCount="693">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1065" uniqueCount="641">
   <si>
     <t>SKU</t>
   </si>
@@ -1543,13 +1543,7 @@
     <t>Galvanizado</t>
   </si>
   <si>
-    <t>CLI-11-B-9016-01</t>
-  </si>
-  <si>
-    <t>CLI-P13704-101</t>
-  </si>
-  <si>
-    <t>CLI-P13704-091</t>
+    <t>ISSIV00099</t>
   </si>
   <si>
     <t>SWB00319</t>
@@ -1558,541 +1552,391 @@
     <t>SWB01125</t>
   </si>
   <si>
-    <t>CLI-12-A-6200-02</t>
-  </si>
-  <si>
-    <t>CLI-12-A-6359-02</t>
-  </si>
-  <si>
-    <t>CLI-12-C-6017-01</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6047-03</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6063-06</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6078-05</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6080-06</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6081-06</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6082-05</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6082-06</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6083-06</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6091-03</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6091-08</t>
-  </si>
-  <si>
-    <t>CLI-17-D-6004-01</t>
-  </si>
-  <si>
-    <t>CLI-17-D-6004-02</t>
-  </si>
-  <si>
-    <t>CLI-P13549-16</t>
-  </si>
-  <si>
-    <t>CLI-P13704-151</t>
-  </si>
-  <si>
-    <t>CLI-P13704-152</t>
-  </si>
-  <si>
-    <t>CLI-P17690-17</t>
-  </si>
-  <si>
-    <t>CLI-P19495-01</t>
-  </si>
-  <si>
-    <t>CLI-P19500-16</t>
-  </si>
-  <si>
-    <t>CLI-PP12535-01</t>
-  </si>
-  <si>
-    <t>CLI-PP19152-021</t>
-  </si>
-  <si>
-    <t>CLI-PP19152-031</t>
-  </si>
-  <si>
-    <t>CLI-PP22120-01</t>
-  </si>
-  <si>
-    <t>CLI-PP22121-02</t>
-  </si>
-  <si>
-    <t>CLI-PP7517-10</t>
-  </si>
-  <si>
-    <t>CLI-PP7533-05</t>
-  </si>
-  <si>
-    <t>CLI-PP9247</t>
-  </si>
-  <si>
-    <t>CLI-PP21340-03</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6106-08</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6091-06</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6085-06</t>
-  </si>
-  <si>
-    <t>CLI-P19504-09</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6348-12</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6106-07</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6091-04</t>
-  </si>
-  <si>
-    <t>CLI-17-D-6007-01</t>
-  </si>
-  <si>
-    <t>CLI-17-D-6007-02</t>
-  </si>
-  <si>
-    <t>CLI-17-D-6025-04</t>
-  </si>
-  <si>
-    <t>CLI-12-6010-01</t>
-  </si>
-  <si>
-    <t>CLI-12-6010-03</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6088-08</t>
-  </si>
-  <si>
-    <t>CLI-12-C-6210-02</t>
-  </si>
-  <si>
-    <t>CLI-PP1510-02</t>
-  </si>
-  <si>
-    <t>CLI-PP21340-02</t>
-  </si>
-  <si>
-    <t>CLI-P6298-051</t>
-  </si>
-  <si>
-    <t>CLI-PP22124-01</t>
-  </si>
-  <si>
-    <t>CLI-11-D-3408-01</t>
-  </si>
-  <si>
-    <t>CLI-12-6010-02</t>
-  </si>
-  <si>
-    <t>CLI-12-6010-09</t>
-  </si>
-  <si>
-    <t>CLI-12-6010-10</t>
-  </si>
-  <si>
-    <t>CLI-12-6113-05</t>
-  </si>
-  <si>
-    <t>CLI-12-A-6199-02</t>
-  </si>
-  <si>
-    <t>CLI-12-A-6200-03</t>
-  </si>
-  <si>
-    <t>CLI-12-C-6210-01</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6033-05</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6107-01</t>
-  </si>
-  <si>
-    <t>CLI-P19500-20</t>
-  </si>
-  <si>
-    <t>CLI-P19500-25</t>
-  </si>
-  <si>
-    <t>CLI-P19500-26</t>
-  </si>
-  <si>
-    <t>CLI-P20365-02</t>
-  </si>
-  <si>
-    <t>CLI-PP14805-04</t>
-  </si>
-  <si>
-    <t>CLI-PP15509</t>
-  </si>
-  <si>
-    <t>CLI-PP15536-02</t>
-  </si>
-  <si>
-    <t>CLI-PP17250-06</t>
-  </si>
-  <si>
-    <t>CLI-PP19152-04</t>
-  </si>
-  <si>
-    <t>CLI-PP21340-01</t>
-  </si>
-  <si>
-    <t>CLI-PP22121-01</t>
-  </si>
-  <si>
-    <t>CLI-11-7761-02</t>
-  </si>
-  <si>
-    <t>CLI-11-7761-03</t>
-  </si>
-  <si>
-    <t>CLI-11-7761-04</t>
+    <t>SWB00467</t>
+  </si>
+  <si>
+    <t>SWB00468</t>
+  </si>
+  <si>
+    <t>SWB00469</t>
+  </si>
+  <si>
+    <t>SWB00471</t>
+  </si>
+  <si>
+    <t>SWB00472</t>
+  </si>
+  <si>
+    <t>SWB00856</t>
+  </si>
+  <si>
+    <t>SWB00053</t>
+  </si>
+  <si>
+    <t>SWB00866</t>
+  </si>
+  <si>
+    <t>SWB00052</t>
+  </si>
+  <si>
+    <t>SWB00847</t>
+  </si>
+  <si>
+    <t>SWB00585</t>
+  </si>
+  <si>
+    <t>SWB00858</t>
+  </si>
+  <si>
+    <t>SWB00656</t>
+  </si>
+  <si>
+    <t>SWB00904</t>
+  </si>
+  <si>
+    <t>SWB01773</t>
+  </si>
+  <si>
+    <t>SWB01377</t>
+  </si>
+  <si>
+    <t>SWB01241</t>
+  </si>
+  <si>
+    <t>SWB00481</t>
+  </si>
+  <si>
+    <t>SWB00321</t>
+  </si>
+  <si>
+    <t>SWB00496</t>
+  </si>
+  <si>
+    <t>SWB00480</t>
+  </si>
+  <si>
+    <t>SWB00475</t>
+  </si>
+  <si>
+    <t>SWB00047</t>
+  </si>
+  <si>
+    <t>SWB00857</t>
+  </si>
+  <si>
+    <t>SWB01329</t>
+  </si>
+  <si>
+    <t>SWB01359</t>
+  </si>
+  <si>
+    <t>SWB00436</t>
+  </si>
+  <si>
+    <t>SWB00438</t>
+  </si>
+  <si>
+    <t>SWB01362</t>
+  </si>
+  <si>
+    <t>SWB01130</t>
+  </si>
+  <si>
+    <t>SWB00320</t>
+  </si>
+  <si>
+    <t>SWB00660</t>
+  </si>
+  <si>
+    <t>SWB00685</t>
+  </si>
+  <si>
+    <t>SWB00688</t>
+  </si>
+  <si>
+    <t>SWB01680</t>
+  </si>
+  <si>
+    <t>SWB01315</t>
+  </si>
+  <si>
+    <t>SWB01316</t>
+  </si>
+  <si>
+    <t>SWB01314</t>
+  </si>
+  <si>
+    <t>SWB01333</t>
   </si>
   <si>
     <t>SWB01126</t>
   </si>
   <si>
-    <t>CLI-11-D-3409-02</t>
-  </si>
-  <si>
     <t>SWB01260</t>
   </si>
   <si>
     <t>SWB01407</t>
   </si>
   <si>
-    <t>CLI-12-D-6089-06</t>
-  </si>
-  <si>
-    <t>CLI-PP21341-12</t>
-  </si>
-  <si>
-    <t>CLI-11-C-6119-01</t>
-  </si>
-  <si>
-    <t>CLI-11-D-6192-01</t>
-  </si>
-  <si>
-    <t>CLI-11-D-6193-01</t>
-  </si>
-  <si>
-    <t>CLI-12-6355-03</t>
-  </si>
-  <si>
-    <t>CLI-17-D-6043-02</t>
-  </si>
-  <si>
-    <t>CLI-17-D-6047-01</t>
-  </si>
-  <si>
-    <t>CLI-P19500-17</t>
-  </si>
-  <si>
-    <t>CLI-P19500-18</t>
-  </si>
-  <si>
-    <t>CLI-P19500-19</t>
-  </si>
-  <si>
-    <t>CLI-P20255-02</t>
-  </si>
-  <si>
-    <t>CLI-11-6463-01</t>
-  </si>
-  <si>
-    <t>CLI-11-8232-01</t>
-  </si>
-  <si>
-    <t>CLI-12-6010-05</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6106-06</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6108-01</t>
-  </si>
-  <si>
-    <t>CLI-16-6047-01</t>
-  </si>
-  <si>
-    <t>CLI-PP14023-06</t>
-  </si>
-  <si>
-    <t>CLI-12-C-6211-08</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6086-07</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6099-13</t>
-  </si>
-  <si>
-    <t>CLI-11-A-6015-01</t>
+    <t>SWB01313</t>
+  </si>
+  <si>
+    <t>SWB01134</t>
+  </si>
+  <si>
+    <t>SWB00657</t>
+  </si>
+  <si>
+    <t>SWB00658</t>
+  </si>
+  <si>
+    <t>SWB00659</t>
+  </si>
+  <si>
+    <t>SWB01679</t>
+  </si>
+  <si>
+    <t>SWB01360</t>
+  </si>
+  <si>
+    <t>SWB01801</t>
+  </si>
+  <si>
+    <t>SWB01802</t>
+  </si>
+  <si>
+    <t>SWB00804</t>
+  </si>
+  <si>
+    <t>SWB02088</t>
+  </si>
+  <si>
+    <t>SWB01410</t>
+  </si>
+  <si>
+    <t>SWB01413</t>
+  </si>
+  <si>
+    <t>SWB01414</t>
+  </si>
+  <si>
+    <t>SWB01405</t>
   </si>
   <si>
     <t>SWB01406</t>
   </si>
   <si>
-    <t>CLI-12-C-6210-03</t>
-  </si>
-  <si>
-    <t>CLI-12-C-6211-07</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6080-07</t>
-  </si>
-  <si>
-    <t>CLI-P14345-22</t>
-  </si>
-  <si>
-    <t>CLI-P19657-01</t>
-  </si>
-  <si>
-    <t>CLI-P19657-24</t>
-  </si>
-  <si>
-    <t>CLI-P19657-25</t>
-  </si>
-  <si>
-    <t>CLI-P19657-26</t>
-  </si>
-  <si>
-    <t>CLI-P19671-05</t>
-  </si>
-  <si>
-    <t>CLI-P20321S-08-01</t>
-  </si>
-  <si>
-    <t>CLI-P20325-23</t>
-  </si>
-  <si>
-    <t>CLI-P20336-01</t>
-  </si>
-  <si>
-    <t>CLI-PP10315-01</t>
-  </si>
-  <si>
-    <t>CLI-PP13629-12</t>
-  </si>
-  <si>
-    <t>CLI-PP17250-05</t>
-  </si>
-  <si>
-    <t>CLI-PP19380-03</t>
-  </si>
-  <si>
-    <t>CLI-PP22114-06</t>
-  </si>
-  <si>
-    <t>CLI-P19660-14</t>
-  </si>
-  <si>
-    <t>CLI-PP19568-02</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6101-01</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6101-02</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6101-05</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6101-06</t>
-  </si>
-  <si>
-    <t>CLI-12-D-7930-01</t>
-  </si>
-  <si>
-    <t>CLI-12-D-7930-02</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6085-07</t>
-  </si>
-  <si>
-    <t>CLI-P20330-02</t>
-  </si>
-  <si>
-    <t>CLI-PP8655</t>
-  </si>
-  <si>
-    <t>CLI-P20321-12</t>
+    <t>SWB01409</t>
+  </si>
+  <si>
+    <t>SWB00049</t>
+  </si>
+  <si>
+    <t>SWB01411</t>
+  </si>
+  <si>
+    <t>SWB01417</t>
+  </si>
+  <si>
+    <t>SWB01418</t>
+  </si>
+  <si>
+    <t>SWB01419</t>
+  </si>
+  <si>
+    <t>SWB01420</t>
+  </si>
+  <si>
+    <t>SWB01421</t>
+  </si>
+  <si>
+    <t>SWB01423</t>
+  </si>
+  <si>
+    <t>SWB01424</t>
+  </si>
+  <si>
+    <t>SWB01425</t>
+  </si>
+  <si>
+    <t>SWB01427</t>
+  </si>
+  <si>
+    <t>SWB01428</t>
+  </si>
+  <si>
+    <t>SWB01430</t>
+  </si>
+  <si>
+    <t>SWB01431</t>
+  </si>
+  <si>
+    <t>SWB01964</t>
+  </si>
+  <si>
+    <t>SWB01422</t>
+  </si>
+  <si>
+    <t>SWB01432</t>
+  </si>
+  <si>
+    <t>SWB01412</t>
+  </si>
+  <si>
+    <t>SWB01426</t>
+  </si>
+  <si>
+    <t>ISSIV00672</t>
+  </si>
+  <si>
+    <t>SWB02037</t>
+  </si>
+  <si>
+    <t>SWB02045</t>
+  </si>
+  <si>
+    <t>SWB02052</t>
+  </si>
+  <si>
+    <t>SWB02038</t>
+  </si>
+  <si>
+    <t>SWB02030</t>
+  </si>
+  <si>
+    <t>SWB02031</t>
+  </si>
+  <si>
+    <t>SWB02039</t>
+  </si>
+  <si>
+    <t>SWB02040</t>
+  </si>
+  <si>
+    <t>SWB02048</t>
+  </si>
+  <si>
+    <t>SWB02049</t>
   </si>
   <si>
     <t>SWB02034</t>
   </si>
   <si>
-    <t>CLI-PP14112-19</t>
-  </si>
-  <si>
-    <t>CLI-P20321-13</t>
-  </si>
-  <si>
-    <t>CLI-11-A-6037-01</t>
-  </si>
-  <si>
-    <t>CLI-11-D-6165-01</t>
-  </si>
-  <si>
-    <t>CLI-P20321-15-11</t>
-  </si>
-  <si>
-    <t>CLI-P20321-15-12</t>
-  </si>
-  <si>
-    <t>CLI-P20512-08</t>
-  </si>
-  <si>
-    <t>CLI-P20512-09</t>
-  </si>
-  <si>
-    <t>CLI-13-D-6196-01</t>
-  </si>
-  <si>
-    <t>CLI-P20512-18</t>
-  </si>
-  <si>
-    <t>CLI-13-D-6195-01</t>
-  </si>
-  <si>
-    <t>CLI-P20512-06</t>
-  </si>
-  <si>
-    <t>CLI-P20512-07</t>
-  </si>
-  <si>
-    <t>CLI-P17311-17</t>
-  </si>
-  <si>
-    <t>CLI-P20321-21</t>
-  </si>
-  <si>
-    <t>CLI-PP20205-121</t>
-  </si>
-  <si>
-    <t>CLI-11-A-6030-01</t>
-  </si>
-  <si>
-    <t>CLI-PP20204-06</t>
-  </si>
-  <si>
-    <t>CLI-PP20203-06</t>
-  </si>
-  <si>
-    <t>CLI-PP20205-061</t>
-  </si>
-  <si>
-    <t>SWB02015</t>
-  </si>
-  <si>
-    <t>SWB02032</t>
-  </si>
-  <si>
-    <t>CLI-P20321S-06</t>
-  </si>
-  <si>
-    <t>CLI-12-6383-01</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6015-05</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6017-02</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6234-08</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6234-06</t>
-  </si>
-  <si>
-    <t>CLI-PP20204-12</t>
-  </si>
-  <si>
-    <t>CLI-PP20204-13</t>
-  </si>
-  <si>
-    <t>CLI-PP20203-12</t>
-  </si>
-  <si>
-    <t>CLI-PP20203-13</t>
-  </si>
-  <si>
-    <t>CLI-PP13949-04</t>
-  </si>
-  <si>
-    <t>CLI-PP13949-09</t>
-  </si>
-  <si>
-    <t>CLI-PP20205-131</t>
-  </si>
-  <si>
-    <t>CLI-PP20205-132</t>
-  </si>
-  <si>
-    <t>CLI-12-6267-01</t>
-  </si>
-  <si>
-    <t>CLI-PP13949-10</t>
-  </si>
-  <si>
-    <t>CLI-PP13949-08</t>
-  </si>
-  <si>
-    <t>CLI-96-6183-01</t>
-  </si>
-  <si>
-    <t>CLI-96-6183-02</t>
-  </si>
-  <si>
-    <t>CLI-P19663-24</t>
-  </si>
-  <si>
-    <t>CLI-12-6265-01</t>
-  </si>
-  <si>
-    <t>CLI-12-D-6234-10</t>
-  </si>
-  <si>
-    <t>CLI-PP22114-05</t>
-  </si>
-  <si>
-    <t>CLI-PP7517-01</t>
-  </si>
-  <si>
-    <t>CLI-P20325-25</t>
-  </si>
-  <si>
-    <t>CLI-P20325-24</t>
-  </si>
-  <si>
-    <t>CLI-P14734-10</t>
+    <t>SWB02050</t>
+  </si>
+  <si>
+    <t>SWB02033</t>
+  </si>
+  <si>
+    <t>SWB02046</t>
+  </si>
+  <si>
+    <t>SWB02047</t>
+  </si>
+  <si>
+    <t>SWB02035</t>
+  </si>
+  <si>
+    <t>SWB02041</t>
+  </si>
+  <si>
+    <t>SWB01526</t>
+  </si>
+  <si>
+    <t>SWB02029</t>
+  </si>
+  <si>
+    <t>SWB02054</t>
+  </si>
+  <si>
+    <t>SWB02053</t>
+  </si>
+  <si>
+    <t>SWB02055</t>
+  </si>
+  <si>
+    <t>SWB02036</t>
+  </si>
+  <si>
+    <t>SWB02042</t>
+  </si>
+  <si>
+    <t>SWB02043</t>
+  </si>
+  <si>
+    <t>SWB01944</t>
+  </si>
+  <si>
+    <t>SWB00456</t>
+  </si>
+  <si>
+    <t>SWB01167</t>
+  </si>
+  <si>
+    <t>SWB01169</t>
+  </si>
+  <si>
+    <t>SWB00488</t>
+  </si>
+  <si>
+    <t>SWB01524</t>
+  </si>
+  <si>
+    <t>SWB01525</t>
+  </si>
+  <si>
+    <t>SWB01522</t>
+  </si>
+  <si>
+    <t>SWB01523</t>
+  </si>
+  <si>
+    <t>SWB01515</t>
+  </si>
+  <si>
+    <t>SWB01517</t>
+  </si>
+  <si>
+    <t>SWB01528</t>
+  </si>
+  <si>
+    <t>SWB01529</t>
+  </si>
+  <si>
+    <t>SWB01162</t>
+  </si>
+  <si>
+    <t>SWB01518</t>
+  </si>
+  <si>
+    <t>SWB02051</t>
+  </si>
+  <si>
+    <t>SWB01469</t>
+  </si>
+  <si>
+    <t>SWB01311</t>
+  </si>
+  <si>
+    <t>SWB01487</t>
+  </si>
+  <si>
+    <t>SWB01161</t>
+  </si>
+  <si>
+    <t>SWB01433</t>
+  </si>
+  <si>
+    <t>SWB01378</t>
+  </si>
+  <si>
+    <t>SWB02437</t>
+  </si>
+  <si>
+    <t>SWB02436</t>
+  </si>
+  <si>
+    <t>SWB00589</t>
   </si>
 </sst>
 </file>
@@ -2484,7 +2328,7 @@
         <v>507</v>
       </c>
       <c r="F3" t="s">
-        <v>510</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:6">
@@ -2504,7 +2348,7 @@
         <v>507</v>
       </c>
       <c r="F4" t="s">
-        <v>511</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5" spans="1:6">
@@ -2524,7 +2368,7 @@
         <v>507</v>
       </c>
       <c r="F5" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
     </row>
     <row r="6" spans="1:6">
@@ -2544,7 +2388,7 @@
         <v>507</v>
       </c>
       <c r="F6" t="s">
-        <v>513</v>
+        <v>511</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -2564,7 +2408,7 @@
         <v>507</v>
       </c>
       <c r="F7" t="s">
-        <v>514</v>
+        <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:6">
@@ -2584,7 +2428,7 @@
         <v>507</v>
       </c>
       <c r="F8" t="s">
-        <v>515</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:6">
@@ -2604,7 +2448,7 @@
         <v>507</v>
       </c>
       <c r="F9" t="s">
-        <v>516</v>
+        <v>13</v>
       </c>
     </row>
     <row r="10" spans="1:6">
@@ -2624,7 +2468,7 @@
         <v>507</v>
       </c>
       <c r="F10" t="s">
-        <v>517</v>
+        <v>512</v>
       </c>
     </row>
     <row r="11" spans="1:6">
@@ -2644,7 +2488,7 @@
         <v>507</v>
       </c>
       <c r="F11" t="s">
-        <v>518</v>
+        <v>513</v>
       </c>
     </row>
     <row r="12" spans="1:6">
@@ -2664,7 +2508,7 @@
         <v>507</v>
       </c>
       <c r="F12" t="s">
-        <v>519</v>
+        <v>514</v>
       </c>
     </row>
     <row r="13" spans="1:6">
@@ -2684,7 +2528,7 @@
         <v>507</v>
       </c>
       <c r="F13" t="s">
-        <v>520</v>
+        <v>515</v>
       </c>
     </row>
     <row r="14" spans="1:6">
@@ -2704,7 +2548,7 @@
         <v>507</v>
       </c>
       <c r="F14" t="s">
-        <v>521</v>
+        <v>516</v>
       </c>
     </row>
     <row r="15" spans="1:6">
@@ -2724,7 +2568,7 @@
         <v>507</v>
       </c>
       <c r="F15" t="s">
-        <v>522</v>
+        <v>517</v>
       </c>
     </row>
     <row r="16" spans="1:6">
@@ -2744,7 +2588,7 @@
         <v>507</v>
       </c>
       <c r="F16" t="s">
-        <v>523</v>
+        <v>20</v>
       </c>
     </row>
     <row r="17" spans="1:6">
@@ -2764,7 +2608,7 @@
         <v>507</v>
       </c>
       <c r="F17" t="s">
-        <v>524</v>
+        <v>518</v>
       </c>
     </row>
     <row r="18" spans="1:6">
@@ -2784,7 +2628,7 @@
         <v>507</v>
       </c>
       <c r="F18" t="s">
-        <v>525</v>
+        <v>519</v>
       </c>
     </row>
     <row r="19" spans="1:6">
@@ -2804,7 +2648,7 @@
         <v>507</v>
       </c>
       <c r="F19" t="s">
-        <v>526</v>
+        <v>520</v>
       </c>
     </row>
     <row r="20" spans="1:6">
@@ -2824,7 +2668,7 @@
         <v>507</v>
       </c>
       <c r="F20" t="s">
-        <v>527</v>
+        <v>24</v>
       </c>
     </row>
     <row r="21" spans="1:6">
@@ -2844,7 +2688,7 @@
         <v>507</v>
       </c>
       <c r="F21" t="s">
-        <v>528</v>
+        <v>25</v>
       </c>
     </row>
     <row r="22" spans="1:6">
@@ -2864,7 +2708,7 @@
         <v>507</v>
       </c>
       <c r="F22" t="s">
-        <v>529</v>
+        <v>521</v>
       </c>
     </row>
     <row r="23" spans="1:6">
@@ -2884,7 +2728,7 @@
         <v>507</v>
       </c>
       <c r="F23" t="s">
-        <v>530</v>
+        <v>27</v>
       </c>
     </row>
     <row r="24" spans="1:6">
@@ -2904,7 +2748,7 @@
         <v>507</v>
       </c>
       <c r="F24" t="s">
-        <v>531</v>
+        <v>522</v>
       </c>
     </row>
     <row r="25" spans="1:6">
@@ -2924,7 +2768,7 @@
         <v>507</v>
       </c>
       <c r="F25" t="s">
-        <v>532</v>
+        <v>29</v>
       </c>
     </row>
     <row r="26" spans="1:6">
@@ -2944,7 +2788,7 @@
         <v>507</v>
       </c>
       <c r="F26" t="s">
-        <v>533</v>
+        <v>523</v>
       </c>
     </row>
     <row r="27" spans="1:6">
@@ -2964,7 +2808,7 @@
         <v>507</v>
       </c>
       <c r="F27" t="s">
-        <v>534</v>
+        <v>524</v>
       </c>
     </row>
     <row r="28" spans="1:6">
@@ -2984,7 +2828,7 @@
         <v>507</v>
       </c>
       <c r="F28" t="s">
-        <v>535</v>
+        <v>32</v>
       </c>
     </row>
     <row r="29" spans="1:6">
@@ -3004,7 +2848,7 @@
         <v>507</v>
       </c>
       <c r="F29" t="s">
-        <v>536</v>
+        <v>525</v>
       </c>
     </row>
     <row r="30" spans="1:6">
@@ -3024,7 +2868,7 @@
         <v>507</v>
       </c>
       <c r="F30" t="s">
-        <v>537</v>
+        <v>34</v>
       </c>
     </row>
     <row r="31" spans="1:6">
@@ -3044,7 +2888,7 @@
         <v>507</v>
       </c>
       <c r="F31" t="s">
-        <v>538</v>
+        <v>35</v>
       </c>
     </row>
     <row r="32" spans="1:6">
@@ -3064,7 +2908,7 @@
         <v>507</v>
       </c>
       <c r="F32" t="s">
-        <v>539</v>
+        <v>526</v>
       </c>
     </row>
     <row r="33" spans="1:6">
@@ -3084,7 +2928,7 @@
         <v>507</v>
       </c>
       <c r="F33" t="s">
-        <v>540</v>
+        <v>527</v>
       </c>
     </row>
     <row r="34" spans="1:6">
@@ -3104,7 +2948,7 @@
         <v>507</v>
       </c>
       <c r="F34" t="s">
-        <v>541</v>
+        <v>38</v>
       </c>
     </row>
     <row r="35" spans="1:6">
@@ -3124,7 +2968,7 @@
         <v>507</v>
       </c>
       <c r="F35" t="s">
-        <v>542</v>
+        <v>528</v>
       </c>
     </row>
     <row r="36" spans="1:6">
@@ -3144,7 +2988,7 @@
         <v>507</v>
       </c>
       <c r="F36" t="s">
-        <v>543</v>
+        <v>40</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -3164,7 +3008,7 @@
         <v>507</v>
       </c>
       <c r="F37" t="s">
-        <v>544</v>
+        <v>529</v>
       </c>
     </row>
     <row r="38" spans="1:6">
@@ -3184,7 +3028,7 @@
         <v>507</v>
       </c>
       <c r="F38" t="s">
-        <v>545</v>
+        <v>530</v>
       </c>
     </row>
     <row r="39" spans="1:6">
@@ -3204,7 +3048,7 @@
         <v>507</v>
       </c>
       <c r="F39" t="s">
-        <v>546</v>
+        <v>43</v>
       </c>
     </row>
     <row r="40" spans="1:6">
@@ -3224,7 +3068,7 @@
         <v>507</v>
       </c>
       <c r="F40" t="s">
-        <v>547</v>
+        <v>44</v>
       </c>
     </row>
     <row r="41" spans="1:6">
@@ -3244,7 +3088,7 @@
         <v>507</v>
       </c>
       <c r="F41" t="s">
-        <v>548</v>
+        <v>531</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -3264,7 +3108,7 @@
         <v>507</v>
       </c>
       <c r="F42" t="s">
-        <v>549</v>
+        <v>532</v>
       </c>
     </row>
     <row r="43" spans="1:6">
@@ -3284,7 +3128,7 @@
         <v>507</v>
       </c>
       <c r="F43" t="s">
-        <v>550</v>
+        <v>533</v>
       </c>
     </row>
     <row r="44" spans="1:6">
@@ -3304,7 +3148,7 @@
         <v>507</v>
       </c>
       <c r="F44" t="s">
-        <v>551</v>
+        <v>48</v>
       </c>
     </row>
     <row r="45" spans="1:6">
@@ -3324,7 +3168,7 @@
         <v>507</v>
       </c>
       <c r="F45" t="s">
-        <v>552</v>
+        <v>49</v>
       </c>
     </row>
     <row r="46" spans="1:6">
@@ -3344,7 +3188,7 @@
         <v>507</v>
       </c>
       <c r="F46" t="s">
-        <v>553</v>
+        <v>50</v>
       </c>
     </row>
     <row r="47" spans="1:6">
@@ -3364,7 +3208,7 @@
         <v>507</v>
       </c>
       <c r="F47" t="s">
-        <v>554</v>
+        <v>51</v>
       </c>
     </row>
     <row r="48" spans="1:6">
@@ -3384,7 +3228,7 @@
         <v>507</v>
       </c>
       <c r="F48" t="s">
-        <v>555</v>
+        <v>52</v>
       </c>
     </row>
     <row r="49" spans="1:6">
@@ -3404,7 +3248,7 @@
         <v>507</v>
       </c>
       <c r="F49" t="s">
-        <v>556</v>
+        <v>534</v>
       </c>
     </row>
     <row r="50" spans="1:6">
@@ -3424,7 +3268,7 @@
         <v>507</v>
       </c>
       <c r="F50" t="s">
-        <v>557</v>
+        <v>54</v>
       </c>
     </row>
     <row r="51" spans="1:6">
@@ -3444,7 +3288,7 @@
         <v>507</v>
       </c>
       <c r="F51" t="s">
-        <v>558</v>
+        <v>55</v>
       </c>
     </row>
     <row r="52" spans="1:6">
@@ -3464,7 +3308,7 @@
         <v>507</v>
       </c>
       <c r="F52" t="s">
-        <v>559</v>
+        <v>56</v>
       </c>
     </row>
     <row r="53" spans="1:6">
@@ -3484,7 +3328,7 @@
         <v>507</v>
       </c>
       <c r="F53" t="s">
-        <v>560</v>
+        <v>535</v>
       </c>
     </row>
     <row r="54" spans="1:6">
@@ -3504,7 +3348,7 @@
         <v>507</v>
       </c>
       <c r="F54" t="s">
-        <v>561</v>
+        <v>58</v>
       </c>
     </row>
     <row r="55" spans="1:6">
@@ -3524,7 +3368,7 @@
         <v>507</v>
       </c>
       <c r="F55" t="s">
-        <v>562</v>
+        <v>536</v>
       </c>
     </row>
     <row r="56" spans="1:6">
@@ -3544,7 +3388,7 @@
         <v>507</v>
       </c>
       <c r="F56" t="s">
-        <v>563</v>
+        <v>537</v>
       </c>
     </row>
     <row r="57" spans="1:6">
@@ -3564,7 +3408,7 @@
         <v>507</v>
       </c>
       <c r="F57" t="s">
-        <v>564</v>
+        <v>61</v>
       </c>
     </row>
     <row r="58" spans="1:6">
@@ -3584,7 +3428,7 @@
         <v>507</v>
       </c>
       <c r="F58" t="s">
-        <v>565</v>
+        <v>62</v>
       </c>
     </row>
     <row r="59" spans="1:6">
@@ -3604,7 +3448,7 @@
         <v>507</v>
       </c>
       <c r="F59" t="s">
-        <v>566</v>
+        <v>63</v>
       </c>
     </row>
     <row r="60" spans="1:6">
@@ -3624,7 +3468,7 @@
         <v>507</v>
       </c>
       <c r="F60" t="s">
-        <v>567</v>
+        <v>538</v>
       </c>
     </row>
     <row r="61" spans="1:6">
@@ -3644,7 +3488,7 @@
         <v>507</v>
       </c>
       <c r="F61" t="s">
-        <v>568</v>
+        <v>539</v>
       </c>
     </row>
     <row r="62" spans="1:6">
@@ -3664,7 +3508,7 @@
         <v>507</v>
       </c>
       <c r="F62" t="s">
-        <v>569</v>
+        <v>540</v>
       </c>
     </row>
     <row r="63" spans="1:6">
@@ -3684,7 +3528,7 @@
         <v>507</v>
       </c>
       <c r="F63" t="s">
-        <v>570</v>
+        <v>541</v>
       </c>
     </row>
     <row r="64" spans="1:6">
@@ -3704,7 +3548,7 @@
         <v>507</v>
       </c>
       <c r="F64" t="s">
-        <v>571</v>
+        <v>542</v>
       </c>
     </row>
     <row r="65" spans="1:6">
@@ -3724,7 +3568,7 @@
         <v>507</v>
       </c>
       <c r="F65" t="s">
-        <v>572</v>
+        <v>543</v>
       </c>
     </row>
     <row r="66" spans="1:6">
@@ -3744,7 +3588,7 @@
         <v>507</v>
       </c>
       <c r="F66" t="s">
-        <v>573</v>
+        <v>70</v>
       </c>
     </row>
     <row r="67" spans="1:6">
@@ -3764,7 +3608,7 @@
         <v>507</v>
       </c>
       <c r="F67" t="s">
-        <v>574</v>
+        <v>71</v>
       </c>
     </row>
     <row r="68" spans="1:6">
@@ -3784,7 +3628,7 @@
         <v>507</v>
       </c>
       <c r="F68" t="s">
-        <v>575</v>
+        <v>72</v>
       </c>
     </row>
     <row r="69" spans="1:6">
@@ -3804,7 +3648,7 @@
         <v>507</v>
       </c>
       <c r="F69" t="s">
-        <v>576</v>
+        <v>544</v>
       </c>
     </row>
     <row r="70" spans="1:6">
@@ -3824,7 +3668,7 @@
         <v>507</v>
       </c>
       <c r="F70" t="s">
-        <v>577</v>
+        <v>545</v>
       </c>
     </row>
     <row r="71" spans="1:6">
@@ -3844,7 +3688,7 @@
         <v>507</v>
       </c>
       <c r="F71" t="s">
-        <v>578</v>
+        <v>75</v>
       </c>
     </row>
     <row r="72" spans="1:6">
@@ -3864,7 +3708,7 @@
         <v>507</v>
       </c>
       <c r="F72" t="s">
-        <v>579</v>
+        <v>76</v>
       </c>
     </row>
     <row r="73" spans="1:6">
@@ -3884,7 +3728,7 @@
         <v>507</v>
       </c>
       <c r="F73" t="s">
-        <v>580</v>
+        <v>546</v>
       </c>
     </row>
     <row r="74" spans="1:6">
@@ -3904,7 +3748,7 @@
         <v>507</v>
       </c>
       <c r="F74" t="s">
-        <v>581</v>
+        <v>547</v>
       </c>
     </row>
     <row r="75" spans="1:6">
@@ -3924,7 +3768,7 @@
         <v>507</v>
       </c>
       <c r="F75" t="s">
-        <v>582</v>
+        <v>79</v>
       </c>
     </row>
     <row r="76" spans="1:6">
@@ -3944,7 +3788,7 @@
         <v>507</v>
       </c>
       <c r="F76" t="s">
-        <v>583</v>
+        <v>548</v>
       </c>
     </row>
     <row r="77" spans="1:6">
@@ -3964,7 +3808,7 @@
         <v>507</v>
       </c>
       <c r="F77" t="s">
-        <v>584</v>
+        <v>549</v>
       </c>
     </row>
     <row r="78" spans="1:6">
@@ -3984,7 +3828,7 @@
         <v>507</v>
       </c>
       <c r="F78" t="s">
-        <v>585</v>
+        <v>550</v>
       </c>
     </row>
     <row r="79" spans="1:6">
@@ -4004,7 +3848,7 @@
         <v>507</v>
       </c>
       <c r="F79" t="s">
-        <v>586</v>
+        <v>551</v>
       </c>
     </row>
     <row r="80" spans="1:6">
@@ -4024,7 +3868,7 @@
         <v>507</v>
       </c>
       <c r="F80" t="s">
-        <v>587</v>
+        <v>84</v>
       </c>
     </row>
     <row r="81" spans="1:6">
@@ -4044,7 +3888,7 @@
         <v>507</v>
       </c>
       <c r="F81" t="s">
-        <v>588</v>
+        <v>552</v>
       </c>
     </row>
     <row r="82" spans="1:6">
@@ -4064,7 +3908,7 @@
         <v>507</v>
       </c>
       <c r="F82" t="s">
-        <v>589</v>
+        <v>553</v>
       </c>
     </row>
     <row r="83" spans="1:6">
@@ -4084,7 +3928,7 @@
         <v>507</v>
       </c>
       <c r="F83" t="s">
-        <v>590</v>
+        <v>87</v>
       </c>
     </row>
     <row r="84" spans="1:6">
@@ -4104,7 +3948,7 @@
         <v>507</v>
       </c>
       <c r="F84" t="s">
-        <v>591</v>
+        <v>88</v>
       </c>
     </row>
     <row r="85" spans="1:6">
@@ -4124,7 +3968,7 @@
         <v>507</v>
       </c>
       <c r="F85" t="s">
-        <v>592</v>
+        <v>89</v>
       </c>
     </row>
     <row r="86" spans="1:6">
@@ -4144,7 +3988,7 @@
         <v>507</v>
       </c>
       <c r="F86" t="s">
-        <v>593</v>
+        <v>90</v>
       </c>
     </row>
     <row r="87" spans="1:6">
@@ -4164,7 +4008,7 @@
         <v>507</v>
       </c>
       <c r="F87" t="s">
-        <v>594</v>
+        <v>91</v>
       </c>
     </row>
     <row r="88" spans="1:6">
@@ -4184,7 +4028,7 @@
         <v>507</v>
       </c>
       <c r="F88" t="s">
-        <v>595</v>
+        <v>554</v>
       </c>
     </row>
     <row r="89" spans="1:6">
@@ -4204,7 +4048,7 @@
         <v>507</v>
       </c>
       <c r="F89" t="s">
-        <v>596</v>
+        <v>93</v>
       </c>
     </row>
     <row r="90" spans="1:6">
@@ -4224,7 +4068,7 @@
         <v>507</v>
       </c>
       <c r="F90" t="s">
-        <v>597</v>
+        <v>555</v>
       </c>
     </row>
     <row r="91" spans="1:6">
@@ -4244,7 +4088,7 @@
         <v>507</v>
       </c>
       <c r="F91" t="s">
-        <v>598</v>
+        <v>556</v>
       </c>
     </row>
     <row r="92" spans="1:6">
@@ -4264,7 +4108,7 @@
         <v>507</v>
       </c>
       <c r="F92" t="s">
-        <v>599</v>
+        <v>557</v>
       </c>
     </row>
     <row r="93" spans="1:6">
@@ -4284,7 +4128,7 @@
         <v>507</v>
       </c>
       <c r="F93" t="s">
-        <v>600</v>
+        <v>558</v>
       </c>
     </row>
     <row r="94" spans="1:6">
@@ -4304,7 +4148,7 @@
         <v>507</v>
       </c>
       <c r="F94" t="s">
-        <v>601</v>
+        <v>559</v>
       </c>
     </row>
     <row r="95" spans="1:6">
@@ -4324,7 +4168,7 @@
         <v>507</v>
       </c>
       <c r="F95" t="s">
-        <v>602</v>
+        <v>99</v>
       </c>
     </row>
     <row r="96" spans="1:6">
@@ -4344,7 +4188,7 @@
         <v>507</v>
       </c>
       <c r="F96" t="s">
-        <v>603</v>
+        <v>100</v>
       </c>
     </row>
     <row r="97" spans="1:6">
@@ -4364,7 +4208,7 @@
         <v>507</v>
       </c>
       <c r="F97" t="s">
-        <v>604</v>
+        <v>560</v>
       </c>
     </row>
     <row r="98" spans="1:6">
@@ -4384,7 +4228,7 @@
         <v>507</v>
       </c>
       <c r="F98" t="s">
-        <v>605</v>
+        <v>561</v>
       </c>
     </row>
     <row r="99" spans="1:6">
@@ -4404,7 +4248,7 @@
         <v>507</v>
       </c>
       <c r="F99" t="s">
-        <v>606</v>
+        <v>562</v>
       </c>
     </row>
     <row r="100" spans="1:6">
@@ -4424,7 +4268,7 @@
         <v>507</v>
       </c>
       <c r="F100" t="s">
-        <v>607</v>
+        <v>563</v>
       </c>
     </row>
     <row r="101" spans="1:6">
@@ -4444,7 +4288,7 @@
         <v>507</v>
       </c>
       <c r="F101" t="s">
-        <v>608</v>
+        <v>564</v>
       </c>
     </row>
     <row r="102" spans="1:6">
@@ -4464,7 +4308,7 @@
         <v>507</v>
       </c>
       <c r="F102" t="s">
-        <v>609</v>
+        <v>565</v>
       </c>
     </row>
     <row r="103" spans="1:6">
@@ -4484,7 +4328,7 @@
         <v>507</v>
       </c>
       <c r="F103" t="s">
-        <v>610</v>
+        <v>566</v>
       </c>
     </row>
     <row r="104" spans="1:6">
@@ -4504,7 +4348,7 @@
         <v>507</v>
       </c>
       <c r="F104" t="s">
-        <v>611</v>
+        <v>567</v>
       </c>
     </row>
     <row r="105" spans="1:6">
@@ -4524,7 +4368,7 @@
         <v>507</v>
       </c>
       <c r="F105" t="s">
-        <v>612</v>
+        <v>568</v>
       </c>
     </row>
     <row r="106" spans="1:6">
@@ -4544,7 +4388,7 @@
         <v>507</v>
       </c>
       <c r="F106" t="s">
-        <v>613</v>
+        <v>569</v>
       </c>
     </row>
     <row r="107" spans="1:6">
@@ -4564,7 +4408,7 @@
         <v>507</v>
       </c>
       <c r="F107" t="s">
-        <v>614</v>
+        <v>570</v>
       </c>
     </row>
     <row r="108" spans="1:6">
@@ -4584,7 +4428,7 @@
         <v>507</v>
       </c>
       <c r="F108" t="s">
-        <v>615</v>
+        <v>571</v>
       </c>
     </row>
     <row r="109" spans="1:6">
@@ -4604,7 +4448,7 @@
         <v>507</v>
       </c>
       <c r="F109" t="s">
-        <v>616</v>
+        <v>572</v>
       </c>
     </row>
     <row r="110" spans="1:6">
@@ -4624,7 +4468,7 @@
         <v>507</v>
       </c>
       <c r="F110" t="s">
-        <v>617</v>
+        <v>573</v>
       </c>
     </row>
     <row r="111" spans="1:6">
@@ -4644,7 +4488,7 @@
         <v>507</v>
       </c>
       <c r="F111" t="s">
-        <v>618</v>
+        <v>574</v>
       </c>
     </row>
     <row r="112" spans="1:6">
@@ -4664,7 +4508,7 @@
         <v>507</v>
       </c>
       <c r="F112" t="s">
-        <v>619</v>
+        <v>575</v>
       </c>
     </row>
     <row r="113" spans="1:6">
@@ -4684,7 +4528,7 @@
         <v>507</v>
       </c>
       <c r="F113" t="s">
-        <v>620</v>
+        <v>576</v>
       </c>
     </row>
     <row r="114" spans="1:6">
@@ -4704,7 +4548,7 @@
         <v>507</v>
       </c>
       <c r="F114" t="s">
-        <v>621</v>
+        <v>577</v>
       </c>
     </row>
     <row r="115" spans="1:6">
@@ -4724,7 +4568,7 @@
         <v>507</v>
       </c>
       <c r="F115" t="s">
-        <v>622</v>
+        <v>578</v>
       </c>
     </row>
     <row r="116" spans="1:6">
@@ -4744,7 +4588,7 @@
         <v>507</v>
       </c>
       <c r="F116" t="s">
-        <v>623</v>
+        <v>579</v>
       </c>
     </row>
     <row r="117" spans="1:6">
@@ -4764,7 +4608,7 @@
         <v>507</v>
       </c>
       <c r="F117" t="s">
-        <v>624</v>
+        <v>580</v>
       </c>
     </row>
     <row r="118" spans="1:6">
@@ -4784,7 +4628,7 @@
         <v>507</v>
       </c>
       <c r="F118" t="s">
-        <v>625</v>
+        <v>581</v>
       </c>
     </row>
     <row r="119" spans="1:6">
@@ -4804,7 +4648,7 @@
         <v>507</v>
       </c>
       <c r="F119" t="s">
-        <v>626</v>
+        <v>582</v>
       </c>
     </row>
     <row r="120" spans="1:6">
@@ -4824,7 +4668,7 @@
         <v>507</v>
       </c>
       <c r="F120" t="s">
-        <v>627</v>
+        <v>583</v>
       </c>
     </row>
     <row r="121" spans="1:6">
@@ -4844,7 +4688,7 @@
         <v>507</v>
       </c>
       <c r="F121" t="s">
-        <v>628</v>
+        <v>125</v>
       </c>
     </row>
     <row r="122" spans="1:6">
@@ -4864,7 +4708,7 @@
         <v>507</v>
       </c>
       <c r="F122" t="s">
-        <v>629</v>
+        <v>584</v>
       </c>
     </row>
     <row r="123" spans="1:6">
@@ -4884,7 +4728,7 @@
         <v>507</v>
       </c>
       <c r="F123" t="s">
-        <v>630</v>
+        <v>585</v>
       </c>
     </row>
     <row r="124" spans="1:6">
@@ -4904,7 +4748,7 @@
         <v>507</v>
       </c>
       <c r="F124" t="s">
-        <v>631</v>
+        <v>586</v>
       </c>
     </row>
     <row r="125" spans="1:6">
@@ -4924,7 +4768,7 @@
         <v>507</v>
       </c>
       <c r="F125" t="s">
-        <v>632</v>
+        <v>587</v>
       </c>
     </row>
     <row r="126" spans="1:6">
@@ -4944,7 +4788,7 @@
         <v>507</v>
       </c>
       <c r="F126" t="s">
-        <v>633</v>
+        <v>130</v>
       </c>
     </row>
     <row r="127" spans="1:6">
@@ -4964,7 +4808,7 @@
         <v>507</v>
       </c>
       <c r="F127" t="s">
-        <v>634</v>
+        <v>131</v>
       </c>
     </row>
     <row r="128" spans="1:6">
@@ -4984,7 +4828,7 @@
         <v>507</v>
       </c>
       <c r="F128" t="s">
-        <v>635</v>
+        <v>132</v>
       </c>
     </row>
     <row r="129" spans="1:6">
@@ -5004,7 +4848,7 @@
         <v>507</v>
       </c>
       <c r="F129" t="s">
-        <v>636</v>
+        <v>133</v>
       </c>
     </row>
     <row r="130" spans="1:6">
@@ -5024,7 +4868,7 @@
         <v>507</v>
       </c>
       <c r="F130" t="s">
-        <v>637</v>
+        <v>134</v>
       </c>
     </row>
     <row r="131" spans="1:6">
@@ -5044,7 +4888,7 @@
         <v>507</v>
       </c>
       <c r="F131" t="s">
-        <v>638</v>
+        <v>135</v>
       </c>
     </row>
     <row r="132" spans="1:6">
@@ -5064,7 +4908,7 @@
         <v>507</v>
       </c>
       <c r="F132" t="s">
-        <v>639</v>
+        <v>588</v>
       </c>
     </row>
     <row r="133" spans="1:6">
@@ -5084,7 +4928,7 @@
         <v>507</v>
       </c>
       <c r="F133" t="s">
-        <v>640</v>
+        <v>589</v>
       </c>
     </row>
     <row r="134" spans="1:6">
@@ -5104,7 +4948,7 @@
         <v>507</v>
       </c>
       <c r="F134" t="s">
-        <v>641</v>
+        <v>590</v>
       </c>
     </row>
     <row r="135" spans="1:6">
@@ -5121,7 +4965,7 @@
         <v>508</v>
       </c>
       <c r="F135" t="s">
-        <v>642</v>
+        <v>591</v>
       </c>
     </row>
     <row r="136" spans="1:6">
@@ -5138,7 +4982,7 @@
         <v>508</v>
       </c>
       <c r="F136" t="s">
-        <v>643</v>
+        <v>592</v>
       </c>
     </row>
     <row r="137" spans="1:6">
@@ -5155,7 +4999,7 @@
         <v>508</v>
       </c>
       <c r="F137" t="s">
-        <v>644</v>
+        <v>593</v>
       </c>
     </row>
     <row r="138" spans="1:6">
@@ -5172,7 +5016,7 @@
         <v>508</v>
       </c>
       <c r="F138" t="s">
-        <v>645</v>
+        <v>594</v>
       </c>
     </row>
     <row r="139" spans="1:6">
@@ -5189,7 +5033,7 @@
         <v>508</v>
       </c>
       <c r="F139" t="s">
-        <v>646</v>
+        <v>595</v>
       </c>
     </row>
     <row r="140" spans="1:6">
@@ -5206,7 +5050,7 @@
         <v>508</v>
       </c>
       <c r="F140" t="s">
-        <v>647</v>
+        <v>596</v>
       </c>
     </row>
     <row r="141" spans="1:6">
@@ -5223,7 +5067,7 @@
         <v>508</v>
       </c>
       <c r="F141" t="s">
-        <v>648</v>
+        <v>597</v>
       </c>
     </row>
     <row r="142" spans="1:6">
@@ -5240,7 +5084,7 @@
         <v>508</v>
       </c>
       <c r="F142" t="s">
-        <v>649</v>
+        <v>598</v>
       </c>
     </row>
     <row r="143" spans="1:6">
@@ -5257,7 +5101,7 @@
         <v>508</v>
       </c>
       <c r="F143" t="s">
-        <v>650</v>
+        <v>599</v>
       </c>
     </row>
     <row r="144" spans="1:6">
@@ -5274,7 +5118,7 @@
         <v>508</v>
       </c>
       <c r="F144" t="s">
-        <v>651</v>
+        <v>600</v>
       </c>
     </row>
     <row r="145" spans="1:6">
@@ -5291,7 +5135,7 @@
         <v>508</v>
       </c>
       <c r="F145" t="s">
-        <v>652</v>
+        <v>601</v>
       </c>
     </row>
     <row r="146" spans="1:6">
@@ -5308,7 +5152,7 @@
         <v>508</v>
       </c>
       <c r="F146" t="s">
-        <v>653</v>
+        <v>602</v>
       </c>
     </row>
     <row r="147" spans="1:6">
@@ -5325,7 +5169,7 @@
         <v>508</v>
       </c>
       <c r="F147" t="s">
-        <v>654</v>
+        <v>603</v>
       </c>
     </row>
     <row r="148" spans="1:6">
@@ -5342,7 +5186,7 @@
         <v>508</v>
       </c>
       <c r="F148" t="s">
-        <v>655</v>
+        <v>604</v>
       </c>
     </row>
     <row r="149" spans="1:6">
@@ -5359,7 +5203,7 @@
         <v>508</v>
       </c>
       <c r="F149" t="s">
-        <v>656</v>
+        <v>605</v>
       </c>
     </row>
     <row r="150" spans="1:6">
@@ -5376,7 +5220,7 @@
         <v>508</v>
       </c>
       <c r="F150" t="s">
-        <v>657</v>
+        <v>606</v>
       </c>
     </row>
     <row r="151" spans="1:6">
@@ -5393,7 +5237,7 @@
         <v>508</v>
       </c>
       <c r="F151" t="s">
-        <v>658</v>
+        <v>607</v>
       </c>
     </row>
     <row r="152" spans="1:6">
@@ -5410,7 +5254,7 @@
         <v>508</v>
       </c>
       <c r="F152" t="s">
-        <v>659</v>
+        <v>608</v>
       </c>
     </row>
     <row r="153" spans="1:6">
@@ -5427,7 +5271,7 @@
         <v>508</v>
       </c>
       <c r="F153" t="s">
-        <v>660</v>
+        <v>609</v>
       </c>
     </row>
     <row r="154" spans="1:6">
@@ -5444,7 +5288,7 @@
         <v>508</v>
       </c>
       <c r="F154" t="s">
-        <v>661</v>
+        <v>610</v>
       </c>
     </row>
     <row r="155" spans="1:6">
@@ -5461,7 +5305,7 @@
         <v>508</v>
       </c>
       <c r="F155" t="s">
-        <v>662</v>
+        <v>611</v>
       </c>
     </row>
     <row r="156" spans="1:6">
@@ -5478,7 +5322,7 @@
         <v>508</v>
       </c>
       <c r="F156" t="s">
-        <v>663</v>
+        <v>612</v>
       </c>
     </row>
     <row r="157" spans="1:6">
@@ -5495,7 +5339,7 @@
         <v>508</v>
       </c>
       <c r="F157" t="s">
-        <v>664</v>
+        <v>613</v>
       </c>
     </row>
     <row r="158" spans="1:6">
@@ -5512,7 +5356,7 @@
         <v>508</v>
       </c>
       <c r="F158" t="s">
-        <v>665</v>
+        <v>614</v>
       </c>
     </row>
     <row r="159" spans="1:6">
@@ -5529,7 +5373,7 @@
         <v>508</v>
       </c>
       <c r="F159" t="s">
-        <v>666</v>
+        <v>615</v>
       </c>
     </row>
     <row r="160" spans="1:6">
@@ -5546,7 +5390,7 @@
         <v>508</v>
       </c>
       <c r="F160" t="s">
-        <v>667</v>
+        <v>616</v>
       </c>
     </row>
     <row r="161" spans="1:6">
@@ -5563,7 +5407,7 @@
         <v>508</v>
       </c>
       <c r="F161" t="s">
-        <v>668</v>
+        <v>617</v>
       </c>
     </row>
     <row r="162" spans="1:6">
@@ -5580,7 +5424,7 @@
         <v>508</v>
       </c>
       <c r="F162" t="s">
-        <v>669</v>
+        <v>618</v>
       </c>
     </row>
     <row r="163" spans="1:6">
@@ -5597,7 +5441,7 @@
         <v>508</v>
       </c>
       <c r="F163" t="s">
-        <v>670</v>
+        <v>619</v>
       </c>
     </row>
     <row r="164" spans="1:6">
@@ -5614,7 +5458,7 @@
         <v>508</v>
       </c>
       <c r="F164" t="s">
-        <v>671</v>
+        <v>620</v>
       </c>
     </row>
     <row r="165" spans="1:6">
@@ -5631,7 +5475,7 @@
         <v>508</v>
       </c>
       <c r="F165" t="s">
-        <v>672</v>
+        <v>621</v>
       </c>
     </row>
     <row r="166" spans="1:6">
@@ -5648,7 +5492,7 @@
         <v>508</v>
       </c>
       <c r="F166" t="s">
-        <v>673</v>
+        <v>622</v>
       </c>
     </row>
     <row r="167" spans="1:6">
@@ -5665,7 +5509,7 @@
         <v>508</v>
       </c>
       <c r="F167" t="s">
-        <v>674</v>
+        <v>623</v>
       </c>
     </row>
     <row r="168" spans="1:6">
@@ -5682,7 +5526,7 @@
         <v>508</v>
       </c>
       <c r="F168" t="s">
-        <v>675</v>
+        <v>624</v>
       </c>
     </row>
     <row r="169" spans="1:6">
@@ -5699,7 +5543,7 @@
         <v>508</v>
       </c>
       <c r="F169" t="s">
-        <v>676</v>
+        <v>625</v>
       </c>
     </row>
     <row r="170" spans="1:6">
@@ -5716,7 +5560,7 @@
         <v>508</v>
       </c>
       <c r="F170" t="s">
-        <v>677</v>
+        <v>626</v>
       </c>
     </row>
     <row r="171" spans="1:6">
@@ -5733,7 +5577,7 @@
         <v>508</v>
       </c>
       <c r="F171" t="s">
-        <v>678</v>
+        <v>627</v>
       </c>
     </row>
     <row r="172" spans="1:6">
@@ -5750,7 +5594,7 @@
         <v>508</v>
       </c>
       <c r="F172" t="s">
-        <v>679</v>
+        <v>628</v>
       </c>
     </row>
     <row r="173" spans="1:6">
@@ -5767,7 +5611,7 @@
         <v>508</v>
       </c>
       <c r="F173" t="s">
-        <v>680</v>
+        <v>629</v>
       </c>
     </row>
     <row r="174" spans="1:6">
@@ -5784,7 +5628,7 @@
         <v>508</v>
       </c>
       <c r="F174" t="s">
-        <v>681</v>
+        <v>630</v>
       </c>
     </row>
     <row r="175" spans="1:6">
@@ -5801,7 +5645,7 @@
         <v>508</v>
       </c>
       <c r="F175" t="s">
-        <v>682</v>
+        <v>631</v>
       </c>
     </row>
     <row r="176" spans="1:6">
@@ -5818,7 +5662,7 @@
         <v>508</v>
       </c>
       <c r="F176" t="s">
-        <v>683</v>
+        <v>632</v>
       </c>
     </row>
     <row r="177" spans="1:6">
@@ -5835,7 +5679,7 @@
         <v>508</v>
       </c>
       <c r="F177" t="s">
-        <v>684</v>
+        <v>633</v>
       </c>
     </row>
     <row r="178" spans="1:6">
@@ -5852,7 +5696,7 @@
         <v>508</v>
       </c>
       <c r="F178" t="s">
-        <v>685</v>
+        <v>634</v>
       </c>
     </row>
     <row r="179" spans="1:6">
@@ -5869,7 +5713,7 @@
         <v>508</v>
       </c>
       <c r="F179" t="s">
-        <v>686</v>
+        <v>635</v>
       </c>
     </row>
     <row r="180" spans="1:6">
@@ -5889,7 +5733,7 @@
         <v>508</v>
       </c>
       <c r="F180" t="s">
-        <v>687</v>
+        <v>184</v>
       </c>
     </row>
     <row r="181" spans="1:6">
@@ -5909,7 +5753,7 @@
         <v>507</v>
       </c>
       <c r="F181" t="s">
-        <v>688</v>
+        <v>636</v>
       </c>
     </row>
     <row r="182" spans="1:6">
@@ -5929,7 +5773,7 @@
         <v>508</v>
       </c>
       <c r="F182" t="s">
-        <v>689</v>
+        <v>637</v>
       </c>
     </row>
     <row r="183" spans="1:6">
@@ -5949,7 +5793,7 @@
         <v>508</v>
       </c>
       <c r="F183" t="s">
-        <v>690</v>
+        <v>638</v>
       </c>
     </row>
     <row r="184" spans="1:6">
@@ -5969,7 +5813,7 @@
         <v>508</v>
       </c>
       <c r="F184" t="s">
-        <v>691</v>
+        <v>639</v>
       </c>
     </row>
     <row r="185" spans="1:6">
@@ -5989,7 +5833,7 @@
         <v>508</v>
       </c>
       <c r="F185" t="s">
-        <v>692</v>
+        <v>640</v>
       </c>
     </row>
   </sheetData>

</xml_diff>